<commit_message>
mixV xlsx: first sheet = the PNG figure (Excel charts reported broken)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig6_mixV.xlsx
+++ b/figs/data/fig6_mixV.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="그림6 WAF 추이" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="구간별 WAF" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="그림(이미지)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="그림6 WAF 추이" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="구간별 WAF" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1193,6 +1194,36 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="10261282" cy="5104923"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>40</col>
       <colOff>0</colOff>
       <row>1</row>
@@ -1216,7 +1247,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1532,6 +1563,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:AO31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -2308,7 +2353,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Excel charts: marker-only series had both noFill and solidFill in one <a:ln> (Excel removed the drawing); fixed and all xlsx re-checked
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/figs/data/fig6_mixV.xlsx
+++ b/figs/data/fig6_mixV.xlsx
@@ -210,6 +210,49 @@
             </strRef>
           </tx>
           <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
+              <a:solidFill>
+                <a:srgbClr val="2B2A28"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="4"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="2B2A28"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:solidFill>
+                  <a:srgbClr val="2B2A28"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림6 WAF 추이'!$C$2:$C$31</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림6 WAF 추이'!$D$2:$D$31</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'그림6 WAF 추이'!F1</f>
+            </strRef>
+          </tx>
+          <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="34925">
               <a:solidFill>
                 <a:srgbClr val="2A78D6"/>
@@ -234,48 +277,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'그림6 WAF 추이'!$C$2:$C$31</f>
+              <f>'그림6 WAF 추이'!$E$2:$E$31</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'그림6 WAF 추이'!$D$2:$D$31</f>
-            </numRef>
-          </yVal>
-          <smooth val="0"/>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'그림6 WAF 추이'!G1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
-              <a:solidFill>
-                <a:srgbClr val="8A8984"/>
-              </a:solidFill>
-              <a:prstDash val="dash"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <xVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$F$2:$F$3</f>
-            </numRef>
-          </xVal>
-          <yVal>
-            <numRef>
-              <f>'그림6 WAF 추이'!$G$2:$G$3</f>
+              <f>'그림6 WAF 추이'!$F$2:$F$31</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -528,6 +535,42 @@
           <yVal>
             <numRef>
               <f>'그림6 WAF 추이'!$U$2:$U$3</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="10"/>
+          <order val="10"/>
+          <tx>
+            <strRef>
+              <f>'그림6 WAF 추이'!W1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="12700">
+              <a:solidFill>
+                <a:srgbClr val="8A8984"/>
+              </a:solidFill>
+              <a:prstDash val="dash"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'그림6 WAF 추이'!$V$2:$V$3</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'그림6 WAF 추이'!$W$2:$W$3</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -663,6 +706,34 @@
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:srgbClr val="2B2A28"/>
+            </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'구간별 WAF'!$A$2:$A$11</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'구간별 WAF'!$D$2:$D$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'구간별 WAF'!E1</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="2A78D6"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -677,7 +748,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'구간별 WAF'!$D$2:$D$11</f>
+              <f>'구간별 WAF'!$E$2:$E$11</f>
             </numRef>
           </val>
         </ser>
@@ -738,7 +809,7 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>22</col>
+      <col>24</col>
       <colOff>0</colOff>
       <row>1</row>
       <rowOff>0</rowOff>
@@ -1077,7 +1148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W31"/>
+  <dimension ref="A1:Y31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1093,90 +1164,100 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>CAT-47 (최적) 시간(h)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>CAT-47 (최적) 10시간 2.619</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>iCAT-v4 (제안) 시간(h)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>iCAT-v4 (제안) 10시간 2.941</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>→ 2.OLTP x</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>→ 2.OLTP</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>→ 3.Varmail x</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>→ 3.Varmail</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>→ 4.YCSB-A x</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>→ 4.YCSB-A</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>→ 5.YCSB-B x</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>→ 5.YCSB-B</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>→ 6.FIO-Fast x</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>→ 6.FIO-Fast</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>→ 7.Varmail x</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>→ 7.Varmail</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>→ 8.YCSB-A x</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>→ 8.YCSB-A</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>→ 9.OLTP x</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>→ 9.OLTP</t>
         </is>
@@ -1193,54 +1274,60 @@
         <v>0.1667</v>
       </c>
       <c r="D2" t="n">
+        <v>1.1105</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1667</v>
+      </c>
+      <c r="F2" t="n">
         <v>1.1054</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>1.116</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2.239</v>
       </c>
       <c r="I2" t="n">
         <v>0.9</v>
       </c>
       <c r="J2" t="n">
-        <v>3.351</v>
+        <v>2.239</v>
       </c>
       <c r="K2" t="n">
         <v>0.9</v>
       </c>
       <c r="L2" t="n">
-        <v>4.475</v>
+        <v>3.351</v>
       </c>
       <c r="M2" t="n">
         <v>0.9</v>
       </c>
       <c r="N2" t="n">
-        <v>5.593</v>
+        <v>4.475</v>
       </c>
       <c r="O2" t="n">
         <v>0.9</v>
       </c>
       <c r="P2" t="n">
-        <v>6.705</v>
+        <v>5.593</v>
       </c>
       <c r="Q2" t="n">
         <v>0.9</v>
       </c>
       <c r="R2" t="n">
-        <v>7.817</v>
+        <v>6.705</v>
       </c>
       <c r="S2" t="n">
         <v>0.9</v>
       </c>
       <c r="T2" t="n">
+        <v>7.817</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="V2" t="n">
         <v>8.943</v>
       </c>
-      <c r="U2" t="n">
+      <c r="W2" t="n">
         <v>0.9</v>
       </c>
     </row>
@@ -1255,54 +1342,60 @@
         <v>0.5</v>
       </c>
       <c r="D3" t="n">
+        <v>1.0569</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F3" t="n">
         <v>1.0448</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>1.116</v>
-      </c>
-      <c r="G3" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2.239</v>
       </c>
       <c r="I3" t="n">
         <v>5.7</v>
       </c>
       <c r="J3" t="n">
-        <v>3.351</v>
+        <v>2.239</v>
       </c>
       <c r="K3" t="n">
         <v>5.7</v>
       </c>
       <c r="L3" t="n">
-        <v>4.475</v>
+        <v>3.351</v>
       </c>
       <c r="M3" t="n">
         <v>5.7</v>
       </c>
       <c r="N3" t="n">
-        <v>5.593</v>
+        <v>4.475</v>
       </c>
       <c r="O3" t="n">
         <v>5.7</v>
       </c>
       <c r="P3" t="n">
-        <v>6.705</v>
+        <v>5.593</v>
       </c>
       <c r="Q3" t="n">
         <v>5.7</v>
       </c>
       <c r="R3" t="n">
-        <v>7.817</v>
+        <v>6.705</v>
       </c>
       <c r="S3" t="n">
         <v>5.7</v>
       </c>
       <c r="T3" t="n">
+        <v>7.817</v>
+      </c>
+      <c r="U3" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="V3" t="n">
         <v>8.943</v>
       </c>
-      <c r="U3" t="n">
+      <c r="W3" t="n">
         <v>5.7</v>
       </c>
     </row>
@@ -1317,6 +1410,12 @@
         <v>0.8333</v>
       </c>
       <c r="D4" t="n">
+        <v>1.0481</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.8333</v>
+      </c>
+      <c r="F4" t="n">
         <v>1.0363</v>
       </c>
     </row>
@@ -1331,6 +1430,12 @@
         <v>1.1667</v>
       </c>
       <c r="D5" t="n">
+        <v>1.0988</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1.1667</v>
+      </c>
+      <c r="F5" t="n">
         <v>1.076</v>
       </c>
     </row>
@@ -1345,6 +1450,12 @@
         <v>1.5</v>
       </c>
       <c r="D6" t="n">
+        <v>1.1006</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F6" t="n">
         <v>1.0903</v>
       </c>
     </row>
@@ -1359,6 +1470,12 @@
         <v>1.8333</v>
       </c>
       <c r="D7" t="n">
+        <v>1.1002</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1.8333</v>
+      </c>
+      <c r="F7" t="n">
         <v>1.0876</v>
       </c>
     </row>
@@ -1373,6 +1490,12 @@
         <v>2.1667</v>
       </c>
       <c r="D8" t="n">
+        <v>1.9669</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2.1667</v>
+      </c>
+      <c r="F8" t="n">
         <v>2.0645</v>
       </c>
     </row>
@@ -1387,6 +1510,12 @@
         <v>2.5</v>
       </c>
       <c r="D9" t="n">
+        <v>2.5974</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F9" t="n">
         <v>2.699</v>
       </c>
     </row>
@@ -1401,6 +1530,12 @@
         <v>2.8333</v>
       </c>
       <c r="D10" t="n">
+        <v>2.6118</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.8333</v>
+      </c>
+      <c r="F10" t="n">
         <v>2.7236</v>
       </c>
     </row>
@@ -1415,6 +1550,12 @@
         <v>3.1667</v>
       </c>
       <c r="D11" t="n">
+        <v>2.6174</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3.1667</v>
+      </c>
+      <c r="F11" t="n">
         <v>2.7216</v>
       </c>
     </row>
@@ -1429,6 +1570,12 @@
         <v>3.5</v>
       </c>
       <c r="D12" t="n">
+        <v>2.1485</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F12" t="n">
         <v>1.9551</v>
       </c>
     </row>
@@ -1443,6 +1590,12 @@
         <v>3.8333</v>
       </c>
       <c r="D13" t="n">
+        <v>1.0883</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3.8333</v>
+      </c>
+      <c r="F13" t="n">
         <v>1.0766</v>
       </c>
     </row>
@@ -1457,6 +1610,12 @@
         <v>4.1667</v>
       </c>
       <c r="D14" t="n">
+        <v>1.0736</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4.1667</v>
+      </c>
+      <c r="F14" t="n">
         <v>1.0738</v>
       </c>
     </row>
@@ -1471,6 +1630,12 @@
         <v>4.5</v>
       </c>
       <c r="D15" t="n">
+        <v>1.0936</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F15" t="n">
         <v>1.101</v>
       </c>
     </row>
@@ -1485,6 +1650,12 @@
         <v>4.8333</v>
       </c>
       <c r="D16" t="n">
+        <v>1.5088</v>
+      </c>
+      <c r="E16" t="n">
+        <v>4.8333</v>
+      </c>
+      <c r="F16" t="n">
         <v>1.4498</v>
       </c>
     </row>
@@ -1499,6 +1670,12 @@
         <v>5.1667</v>
       </c>
       <c r="D17" t="n">
+        <v>1.4907</v>
+      </c>
+      <c r="E17" t="n">
+        <v>5.1667</v>
+      </c>
+      <c r="F17" t="n">
         <v>1.4737</v>
       </c>
     </row>
@@ -1513,6 +1690,12 @@
         <v>5.5</v>
       </c>
       <c r="D18" t="n">
+        <v>3.5151</v>
+      </c>
+      <c r="E18" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F18" t="n">
         <v>4.2343</v>
       </c>
     </row>
@@ -1527,6 +1710,12 @@
         <v>5.8333</v>
       </c>
       <c r="D19" t="n">
+        <v>3.9377</v>
+      </c>
+      <c r="E19" t="n">
+        <v>5.8333</v>
+      </c>
+      <c r="F19" t="n">
         <v>4.7429</v>
       </c>
     </row>
@@ -1541,6 +1730,12 @@
         <v>6.1667</v>
       </c>
       <c r="D20" t="n">
+        <v>3.9394</v>
+      </c>
+      <c r="E20" t="n">
+        <v>6.1667</v>
+      </c>
+      <c r="F20" t="n">
         <v>4.7476</v>
       </c>
     </row>
@@ -1555,6 +1750,12 @@
         <v>6.5</v>
       </c>
       <c r="D21" t="n">
+        <v>3.9432</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F21" t="n">
         <v>4.7527</v>
       </c>
     </row>
@@ -1569,6 +1770,12 @@
         <v>6.8333</v>
       </c>
       <c r="D22" t="n">
+        <v>3.4273</v>
+      </c>
+      <c r="E22" t="n">
+        <v>6.8333</v>
+      </c>
+      <c r="F22" t="n">
         <v>4.5411</v>
       </c>
     </row>
@@ -1583,6 +1790,12 @@
         <v>7.1667</v>
       </c>
       <c r="D23" t="n">
+        <v>3.2229</v>
+      </c>
+      <c r="E23" t="n">
+        <v>7.1667</v>
+      </c>
+      <c r="F23" t="n">
         <v>4.1879</v>
       </c>
     </row>
@@ -1597,6 +1810,12 @@
         <v>7.5</v>
       </c>
       <c r="D24" t="n">
+        <v>3.1546</v>
+      </c>
+      <c r="E24" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F24" t="n">
         <v>3.7965</v>
       </c>
     </row>
@@ -1611,6 +1830,12 @@
         <v>7.8333</v>
       </c>
       <c r="D25" t="n">
+        <v>3.0093</v>
+      </c>
+      <c r="E25" t="n">
+        <v>7.8333</v>
+      </c>
+      <c r="F25" t="n">
         <v>3.3083</v>
       </c>
     </row>
@@ -1625,6 +1850,12 @@
         <v>8.166700000000001</v>
       </c>
       <c r="D26" t="n">
+        <v>1.1395</v>
+      </c>
+      <c r="E26" t="n">
+        <v>8.166700000000001</v>
+      </c>
+      <c r="F26" t="n">
         <v>1.135</v>
       </c>
     </row>
@@ -1639,6 +1870,12 @@
         <v>8.5</v>
       </c>
       <c r="D27" t="n">
+        <v>1.1532</v>
+      </c>
+      <c r="E27" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F27" t="n">
         <v>1.1274</v>
       </c>
     </row>
@@ -1653,6 +1890,12 @@
         <v>8.833299999999999</v>
       </c>
       <c r="D28" t="n">
+        <v>1.2414</v>
+      </c>
+      <c r="E28" t="n">
+        <v>8.833299999999999</v>
+      </c>
+      <c r="F28" t="n">
         <v>1.2638</v>
       </c>
     </row>
@@ -1667,6 +1910,12 @@
         <v>9.166700000000001</v>
       </c>
       <c r="D29" t="n">
+        <v>1.3211</v>
+      </c>
+      <c r="E29" t="n">
+        <v>9.166700000000001</v>
+      </c>
+      <c r="F29" t="n">
         <v>1.2955</v>
       </c>
     </row>
@@ -1681,11 +1930,17 @@
         <v>9.5</v>
       </c>
       <c r="D30" t="n">
+        <v>1.3451</v>
+      </c>
+      <c r="E30" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F30" t="n">
         <v>1.303</v>
       </c>
-      <c r="W30" t="inlineStr">
-        <is>
-          <t>점선 = 워크로드 전환, 위 글자 = 구간. FIO 파일 5 GiB(차가운 영역 3 GiB), DB 60만, 표 3 준비. 정책마다 1회. CAT-37=두 번째 PC, iCAT-v4=이 PC. YCSB 요청 실패 0건.</t>
+      <c r="Y30" t="inlineStr">
+        <is>
+          <t>점선 = 워크로드 전환, 위 글자 = 구간. FIO 파일 5 GiB(차가운 영역 3 GiB), DB 60만, 표 3 준비. 정책마다 1회. CAT-37=두 번째 PC, CAT-47=이 PC, iCAT-v4=이 PC. YCSB 요청 실패 0건.</t>
         </is>
       </c>
     </row>
@@ -1700,6 +1955,12 @@
         <v>9.833299999999999</v>
       </c>
       <c r="D31" t="n">
+        <v>1.3399</v>
+      </c>
+      <c r="E31" t="n">
+        <v>9.833299999999999</v>
+      </c>
+      <c r="F31" t="n">
         <v>1.3012</v>
       </c>
     </row>
@@ -1715,7 +1976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1723,6 +1984,8 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1743,12 +2006,22 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>CAT-47 (최적)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>iCAT-v4 (제안)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>v4 vs CAT-37 (%)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>v4 vs CAT-47 (%)</t>
         </is>
       </c>
     </row>
@@ -1767,10 +2040,16 @@
         <v>1.06</v>
       </c>
       <c r="D2" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E2" t="n">
         <v>1.064</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0.3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-0.6</v>
       </c>
     </row>
     <row r="3">
@@ -1788,10 +2067,16 @@
         <v>1.135</v>
       </c>
       <c r="D3" t="n">
+        <v>1.102</v>
+      </c>
+      <c r="E3" t="n">
         <v>1.088</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>-4.1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-1.3</v>
       </c>
     </row>
     <row r="4">
@@ -1809,10 +2094,16 @@
         <v>2.817</v>
       </c>
       <c r="D4" t="n">
+        <v>2.599</v>
+      </c>
+      <c r="E4" t="n">
         <v>2.698</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>-4.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>3.8</v>
       </c>
     </row>
     <row r="5">
@@ -1830,10 +2121,16 @@
         <v>1.118</v>
       </c>
       <c r="D5" t="n">
+        <v>1.124</v>
+      </c>
+      <c r="E5" t="n">
         <v>1.144</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>2.4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.8</v>
       </c>
     </row>
     <row r="6">
@@ -1851,10 +2148,16 @@
         <v>1.489</v>
       </c>
       <c r="D6" t="n">
+        <v>1.418</v>
+      </c>
+      <c r="E6" t="n">
         <v>1.412</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>-5.2</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-0.4</v>
       </c>
     </row>
     <row r="7">
@@ -1872,10 +2175,16 @@
         <v>5.189</v>
       </c>
       <c r="D7" t="n">
+        <v>3.934</v>
+      </c>
+      <c r="E7" t="n">
         <v>4.741</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>-8.6</v>
+      </c>
+      <c r="G7" t="n">
+        <v>20.5</v>
       </c>
     </row>
     <row r="8">
@@ -1893,10 +2202,16 @@
         <v>4.339</v>
       </c>
       <c r="D8" t="n">
+        <v>3.232</v>
+      </c>
+      <c r="E8" t="n">
         <v>4.028</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>-7.2</v>
+      </c>
+      <c r="G8" t="n">
+        <v>24.6</v>
       </c>
     </row>
     <row r="9">
@@ -1914,10 +2229,16 @@
         <v>1.174</v>
       </c>
       <c r="D9" t="n">
+        <v>1.196</v>
+      </c>
+      <c r="E9" t="n">
         <v>1.211</v>
       </c>
-      <c r="E9" t="n">
+      <c r="F9" t="n">
         <v>3.2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.3</v>
       </c>
     </row>
     <row r="10">
@@ -1935,10 +2256,16 @@
         <v>1.521</v>
       </c>
       <c r="D10" t="n">
+        <v>1.339</v>
+      </c>
+      <c r="E10" t="n">
         <v>1.309</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>-14</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-2.3</v>
       </c>
     </row>
     <row r="11">
@@ -1952,16 +2279,22 @@
         <v>3.011</v>
       </c>
       <c r="D11" s="1" t="n">
+        <v>2.619</v>
+      </c>
+      <c r="E11" s="1" t="n">
         <v>2.941</v>
       </c>
-      <c r="E11" s="1" t="n">
+      <c r="F11" s="1" t="n">
         <v>-2.3</v>
+      </c>
+      <c r="G11" s="1" t="n">
+        <v>12.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>음수(%) = v4의 WAF가 더 낮음(좋음). FIO 파일 5 GiB(차가운 영역 3 GiB), DB 60만, 표 3 준비. 정책마다 1회. CAT-37=두 번째 PC, iCAT-v4=이 PC. YCSB 요청 실패 0건.</t>
+          <t>음수(%) = v4의 WAF가 더 낮음(좋음). FIO 파일 5 GiB(차가운 영역 3 GiB), DB 60만, 표 3 준비. 정책마다 1회. CAT-37=두 번째 PC, CAT-47=이 PC, iCAT-v4=이 PC. YCSB 요청 실패 0건.</t>
         </is>
       </c>
     </row>

</xml_diff>